<commit_message>
docs: update change tracker (50 items) - PBKDF2, receive/cross-chain ports on all clients, $8.82, builds
</commit_message>
<xml_diff>
--- a/docs/Thanos_Wallet_Change_Tracker.xlsx
+++ b/docs/Thanos_Wallet_Change_Tracker.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Tracker'!$A$3:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Change Tracker'!$A$3:$I$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -540,18 +540,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
     <col width="44" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -564,7 +564,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Updated 2026-06-17  -  Mobile items are in APK build 50086075  -  Web/Landing items are pushed to origin/main and go live on the next web redeploy</t>
+          <t>Updated 2026-06-18  -  Web is LIVE &amp; verified current  -  Mobile in APK build fceaee9b  -  Extension in rebuilt zip 0.2.0</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Token detail: Buy button + circulating supply</t>
+          <t>Token detail: Buy + circulating supply</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Verified existing header switcher works</t>
+          <t>Verified existing header switcher</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>NFTs screen (honest empty state + marketplace)</t>
+          <t>NFTs screen (honest empty + marketplace)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Import-choose + import-pk flow, EVM-gated</t>
+          <t>Import-choose + import-pk flow</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1086,12 +1086,12 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Stuck on 'Encrypting...' after wallet creation</t>
+          <t>Stuck on 'Encrypting' (first Argon2 attempt)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Argon2 19MiB/t2/p1 + vault.kdf unlock</t>
+          <t>Argon2 19MiB (still too slow on weak device)</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>In APK (verified)</t>
+          <t>Superseded by PBKDF2</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -1126,17 +1126,17 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Choose 12 / 24-word phrase length</t>
+          <t>Encryption took 5-10 MIN / app crashed</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>Added create-length step</t>
+          <t>KDF Argon2 -&gt; PBKDF2 600k (~1-3s)</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -1146,12 +1146,12 @@
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>13edfb9</t>
+          <t>4a14a85</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -1176,12 +1176,12 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Onboarding buttons untappable w/ keyboard open</t>
+          <t>Splash light-&gt;dark flash + logo not showing</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>keyboardShouldPersistTaps=handled</t>
+          <t>Dark splash bg (#080809) + userInterfaceStyle dark</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1191,12 +1191,12 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>a7e6571</t>
+          <t>2980848</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -1216,17 +1216,17 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Onboarding usability + dark default + web colors</t>
+          <t>'I understand' / 'Create wallet' buttons wrapped</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Dark-first, palette match, audit fixes</t>
+          <t>numberOfLines + adjustsFontSizeToFit + wider btn</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1236,12 +1236,12 @@
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>ca035c7</t>
+          <t>4a14a85</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1261,17 +1261,17 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Asset</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Discover logos + ecosystem sync (Makalu/Kamet)</t>
+          <t>Choose 12 / 24-word phrase length</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Added entries + Infrastructure section + logos</t>
+          <t>Added create-length step</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1281,12 +1281,12 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>17ff5ea</t>
+          <t>13edfb9</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -1306,17 +1306,17 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>LITHO currency symbol</t>
+          <t>Onboarding buttons untappable w/ keyboard</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Embedded LithoSym font via expo-font plugin</t>
+          <t>keyboardShouldPersistTaps=handled</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1326,12 +1326,12 @@
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>427db10</t>
+          <t>a7e6571</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>In APK 50086075</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -1351,17 +1351,17 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Rebuild APK with all parity features</t>
+          <t>Onboarding usability + dark default + colors</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>EAS build 50086075</t>
+          <t>Dark-first, palette, audit fixes</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1371,12 +1371,12 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>ca035c7</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Delivered (link)</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1386,27 +1386,27 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Asset</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Cosmos Hub send showed LITHO icon</t>
+          <t>Discover logos + ecosystem sync</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Map cosmos-&gt;ATOM + add ATOM logo</t>
+          <t>Makalu/Kamet entries + Infra section + logos</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -1416,12 +1416,12 @@
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>d1c9473</t>
+          <t>17ff5ea</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -1446,12 +1446,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Swap stablecoin pairs w/ fixed rates</t>
+          <t>LITHO currency symbol</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>LAX/USDC.USDT.DAI + stable-stable, Litho-pinned</t>
+          <t>Embedded LithoSym font via expo-font plugin</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1461,12 +1461,12 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>8f76cf7</t>
+          <t>427db10</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1476,27 +1476,27 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Swap full-screen from nav (popup only from Home)</t>
+          <t>Receive: network -&gt; asset -&gt; QR (SafePal)</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>fullScreen Modal variant + entry split</t>
+          <t>Step flow + asset name/logo + coin warning</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1506,12 +1506,12 @@
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>61fc516</t>
+          <t>32739c1</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1521,27 +1521,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Receive flow: select network -&gt; address + QR</t>
+          <t>Cross-chain swap (tabs + chains + recipient)</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Drill-in flow (SafePal/Trust style)</t>
+          <t>Swap/Cross-chain/Bridge tabs, indicative rate</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1551,12 +1551,12 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>d0323e1</t>
+          <t>26002e8</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>In APK fceaee9b</t>
         </is>
       </c>
     </row>
@@ -1581,12 +1581,12 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Discover screen scroll issue</t>
+          <t>Cosmos Hub send showed LITHO icon</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Made Discover scroll (main is overflow:hidden)</t>
+          <t>Map cosmos-&gt;ATOM + add ATOM logo</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -1596,12 +1596,12 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>9ee0eee</t>
+          <t>d1c9473</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -1621,17 +1621,17 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Asset</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Discover logos (Makalu/Kamet/LITHO Deals)</t>
+          <t>Swap stablecoin pairs w/ fixed rates</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Wired client app-icon pack</t>
+          <t>LAX/USDC.USDT.DAI + stable-stable</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -1641,12 +1641,12 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>da8d0aa</t>
+          <t>8f76cf7</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -1666,17 +1666,17 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>LITHO currency symbol</t>
+          <t>Swap full-screen from nav (popup from Home)</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>Bundled single-glyph font + LithoSym component</t>
+          <t>fullScreen Modal variant + entry split</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -1686,12 +1686,12 @@
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>18147e3</t>
+          <t>61fc516</t>
         </is>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -1701,27 +1701,27 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Cross</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Prices from CoinGecko/CMC (non-fixed tokens)</t>
+          <t>Receive: network -&gt; asset -&gt; QR (SafePal)</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>MUSA live via mansa-ai; JOT/BLDR/FGPT not listed</t>
+          <t>Drill-in network-&gt;asset-&gt;QR + asset header</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -1731,12 +1731,12 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>bc0d694</t>
+          <t>159ffe9</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -1746,27 +1746,27 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Cross</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>LITHO fixed price 8.60 -&gt; 8.82</t>
+          <t>Receive preselects network from an asset</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>Updated web/mobile/sdk-core/worker; swap rate corrected</t>
+          <t>Token-detail Receive jumps to that asset's QR</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -1776,12 +1776,12 @@
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>268c4ba</t>
+          <t>949686a</t>
         </is>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -1796,37 +1796,37 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Cross</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>LITHO &amp; LAX prices fixed (not fetched)</t>
+          <t>Discover screen scroll issue</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>LITHO $8.82, LAX peg; ego.exchange noted, no change</t>
-        </is>
-      </c>
-      <c r="G30" s="10" t="inlineStr">
-        <is>
-          <t>Decision</t>
+          <t>Made Discover scroll (main overflow:hidden)</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>4349a55</t>
+          <t>9ee0eee</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Policy</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1836,7 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
@@ -1846,17 +1846,17 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Asset</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>Token detail as full-screen page</t>
+          <t>Discover logos (Makalu/Kamet/LITHO Deals)</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>Trust/SafePal-style full-screen</t>
+          <t>Wired client app-icon pack</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -1866,12 +1866,12 @@
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>99d0dce</t>
+          <t>da8d0aa</t>
         </is>
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -1896,12 +1896,12 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Make swap cross-chain (chain selectors + recipient)</t>
+          <t>LITHO currency symbol (bundled font)</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Swap/Cross-chain/Bridge tabs UI; exec needs MultX bridge (offline)</t>
+          <t>Single-glyph font + LithoSym component</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -1911,12 +1911,12 @@
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>1c94f53</t>
+          <t>18147e3</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Redeploy pending; exec when bridge live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -1931,22 +1931,22 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Landing</t>
+          <t>Cross</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Pricing</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>25% UI increase (125%) on the site</t>
+          <t>Prices from CoinGecko (non-fixed tokens)</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>body zoom 1.1-&gt;1.25 + vh divisors in lockstep</t>
+          <t>MUSA live via mansa-ai; JOT/BLDR/FGPT unlisted</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>a886df9</t>
+          <t>bc0d694</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -1971,27 +1971,27 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Landing</t>
+          <t>Cross</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Pricing</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>125% on the landing on mobile too</t>
+          <t>LITHO fixed price -&gt; $8.82 (LAX $1.0001)</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Mobile-only landing zoom (compounding-safe)</t>
+          <t>Updated web/mobile/sdk-core/worker</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -2001,12 +2001,12 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>977c710</t>
+          <t>268c4ba</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -2016,12 +2016,12 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Landing</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -2031,12 +2031,12 @@
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>APK direct download on thanos.fi</t>
+          <t>Cross-chain swap UI (tabs + chains + recipient)</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t>/download route</t>
+          <t>Swap/Cross-chain/Bridge tabs, live indicative rate</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -2046,12 +2046,12 @@
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>7e1dd1d</t>
+          <t>1c94f53</t>
         </is>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -2061,27 +2061,27 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Landing</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>'Download .apk' card not clickable</t>
+          <t>Token detail as full-screen page</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Android card live -&gt; links to /download</t>
+          <t>Trust/SafePal-style full-screen</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -2091,12 +2091,12 @@
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>b5819fb</t>
+          <t>99d0dce</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -2121,12 +2121,12 @@
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>APK should download as thanos.apk</t>
+          <t>25% UI increase (125%) incl. landing + mobile</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>Stream w/ Content-Disposition filename=thanos.apk</t>
+          <t>body zoom 1.25 + landing mobile zoom</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
@@ -2136,12 +2136,12 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>4f7c6aa</t>
+          <t>a886df9</t>
         </is>
       </c>
       <c r="I37" s="8" t="inlineStr">
         <is>
-          <t>Redeploy pending</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -2151,27 +2151,27 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Landing</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Apply Litho canonical values</t>
+          <t>APK direct download on thanos.fi</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Kamet explorer, IMAGE name, cleanup</t>
+          <t>/download route -&gt; streams thanos.apk</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -2181,12 +2181,12 @@
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>e7cb761</t>
+          <t>7e1dd1d</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -2196,12 +2196,12 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>Landing</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -2211,12 +2211,12 @@
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>Red CI (frozen lockfile + gitleaks)</t>
+          <t>'Download .apk' card not clickable</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>--no-frozen-lockfile + gitleaks allowlist</t>
+          <t>Android card live -&gt; /download</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
@@ -2226,12 +2226,12 @@
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>aa08aed</t>
+          <t>b5819fb</t>
         </is>
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -2241,27 +2241,27 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Landing</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>APK pipeline (lockfile / minify / config)</t>
+          <t>APK downloads as thanos.apk (professional)</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Linux lockfile, R8 off, expo-build-properties</t>
+          <t>Content-Disposition filename=thanos.apk</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -2271,12 +2271,12 @@
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>ecb1d9d+</t>
+          <t>4f7c6aa</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>Resolved</t>
+          <t>LIVE</t>
         </is>
       </c>
     </row>
@@ -2286,47 +2286,587 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Landing</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Point /download at the CURRENT build</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>APK_URL -&gt; build fceaee9b (verified byte-match live)</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>fb22b18</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Web/Ext</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Perf</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Wallet create/unlock took several seconds</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Vault KDF -&gt; native WebCrypto PBKDF2 600k (~100ms)</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>988eab4</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Web LIVE / Ext in zip</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Ext</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Perf</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Extension slow to create/unlock (like the app)</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Argon2 64MiB -&gt; native PBKDF2 600k</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>988eab4</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>In ext zip 0.2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Ext</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Receive: network -&gt; asset -&gt; QR (SafePal)</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Step flow + asset header + coin warning</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>6d6f780</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>In ext zip 0.2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Ext</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Cross-chain swap (tabs + chains + recipient)</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>Swap/Cross-chain/Bridge tabs, indicative rate</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>0ee7a24</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="inlineStr">
+        <is>
+          <t>In ext zip 0.2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Apply Litho canonical values</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Kamet explorer, IMAGE name, cleanup</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>e7cb761</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Red CI (frozen lockfile + gitleaks)</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>--no-frozen-lockfile + gitleaks allowlist</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>aa08aed</t>
+        </is>
+      </c>
+      <c r="I47" s="8" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>APK pipeline (lockfile / minify / config)</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Linux lockfile, R8 off, expo-build-properties</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>ecb1d9d+</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C49" s="8" t="inlineStr">
         <is>
           <t>Cross</t>
         </is>
       </c>
-      <c r="D41" s="8" t="inlineStr">
+      <c r="D49" s="8" t="inlineStr">
         <is>
           <t>Audit</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Confirm production-stage feature set (13 items)</t>
-        </is>
-      </c>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>Verified each vs code; delivered status table</t>
-        </is>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H41" s="8" t="inlineStr">
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Confirm production-stage feature set (13)</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>Verified each vs code; status table</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H49" s="8" t="inlineStr">
         <is>
           <t>audit</t>
         </is>
       </c>
-      <c r="I41" s="8" t="inlineStr">
+      <c r="I49" s="8" t="inlineStr">
         <is>
           <t>Delivered</t>
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Rebuild APK with all fixes + ports</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>EAS build fceaee9b</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Delivered + on thanos.fi/download</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Ext</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Rebuild extension zip</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>wxt zip -&gt; thanosextension-0.2.0-chrome.zip</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="I51" s="8" t="inlineStr">
+        <is>
+          <t>Delivered (6.97 MB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>LITHO &amp; LAX fixed (not fetched)</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>LITHO $8.82, LAX $1.0001; ego.exchange noted</t>
+        </is>
+      </c>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Cross-chain execution gated on MultX bridge</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>UI complete on all clients; exec when bridge live</t>
+        </is>
+      </c>
+      <c r="G53" s="10" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I53" s="8" t="inlineStr">
+        <is>
+          <t>Roadmap (Litho infra)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:I41"/>
+  <autoFilter ref="A3:I53"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -2344,8 +2884,8 @@
   <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2362,7 +2902,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
@@ -2372,23 +2912,23 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Roadmap / separate track</t>
+          <t>Decisions / policy</t>
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Decisions / policy</t>
+          <t>Roadmap</t>
         </is>
       </c>
       <c r="B6" s="13" t="n">
@@ -2402,36 +2942,36 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Mobile delivered in</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>APK build 50086075</t>
+          <t>LIVE &amp; verified current on thanos.fi</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Web/Landing</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>pushed to origin/main - live after web redeploy</t>
+          <t>APK build fceaee9b - install link + on thanos.fi/download</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Redeploy cmd</t>
+          <t>Extension</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>git pull origin main &amp;&amp; docker compose -f docker-compose.yml -f docker-compose.prod.yml up -d --build web</t>
+          <t>rebuilt zip thanosextension-0.2.0-chrome.zip</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2983,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>expo.dev/accounts/imasssad/projects/thanos-wallet/builds/50086075-a78d-4ece-a92e-35c868fcf3a0</t>
+          <t>expo.dev/accounts/imasssad/projects/thanos-wallet/builds/fceaee9b-f3ce-4ab8-b720-a5774643d135</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2995,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Cross-chain swap UI is built; execution unlocks when the MultX bridge backend is online (Litho infra).</t>
+          <t>Cross-chain swap UI done on all 3 clients; execution unlocks when the MultX bridge backend is online (Litho infra).</t>
         </is>
       </c>
     </row>

</xml_diff>